<commit_message>
improve Step7 overview and chart annotations
</commit_message>
<xml_diff>
--- a/config/solvency_taxonomy.xlsx
+++ b/config/solvency_taxonomy.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2672,17 +2672,17 @@
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>AGENT_COUNT</t>
+          <t>RENEWAL_PREMIUM</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>期末个人营销员数量</t>
+          <t>续期签单保费</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>个人营销员数量</t>
+          <t>续期签单保费（万元）</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -2692,17 +2692,17 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>渠道</t>
+          <t>保费</t>
         </is>
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
-          <t>人</t>
+          <t>万元</t>
         </is>
       </c>
       <c r="G44" s="12" t="inlineStr">
         <is>
-          <t>数量</t>
+          <t>金额</t>
         </is>
       </c>
       <c r="H44" s="12" t="inlineStr">
@@ -2712,11 +2712,11 @@
       </c>
       <c r="I44" s="12" t="inlineStr">
         <is>
-          <t>本季度（末）数|本年累计数</t>
-        </is>
-      </c>
-      <c r="J44" s="12" t="str"/>
-      <c r="K44" s="25" t="inlineStr">
+          <t>本季度（末）数|本季度数|本年累计数</t>
+        </is>
+      </c>
+      <c r="J44" s="12" t="inlineStr"/>
+      <c r="K44" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2725,51 +2725,51 @@
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>RISK_RATING</t>
+          <t>AGENT_COUNT</t>
         </is>
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>风险综合评级</t>
+          <t>期末个人营销员数量</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>分类监管评级|风险综合评级结果</t>
+          <t>个人营销员数量</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>风险管理</t>
+          <t>经营指标</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>风险评级</t>
+          <t>渠道</t>
         </is>
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>级</t>
+          <t>人</t>
         </is>
       </c>
       <c r="G45" s="12" t="inlineStr">
         <is>
-          <t>评级</t>
+          <t>数量</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I45" s="12" t="inlineStr">
         <is>
-          <t>本季度数|上季度数</t>
+          <t>本季度（末）数|本年累计数</t>
         </is>
       </c>
       <c r="J45" s="12" t="str"/>
-      <c r="K45" s="31" t="inlineStr">
+      <c r="K45" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2778,37 +2778,37 @@
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>INSURANCE_RISK_CAPITAL</t>
+          <t>RISK_RATING</t>
         </is>
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>寿险业务保险风险最低资本合计</t>
+          <t>风险综合评级</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>保险风险最低资本合计</t>
+          <t>分类监管评级|风险综合评级结果</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>最低资本</t>
+          <t>风险管理</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>保险风险</t>
+          <t>风险评级</t>
         </is>
       </c>
       <c r="F46" s="12" t="inlineStr">
         <is>
-          <t>万元</t>
+          <t>级</t>
         </is>
       </c>
       <c r="G46" s="12" t="inlineStr">
         <is>
-          <t>金额</t>
+          <t>评级</t>
         </is>
       </c>
       <c r="H46" s="12" t="inlineStr">
@@ -2818,11 +2818,11 @@
       </c>
       <c r="I46" s="12" t="inlineStr">
         <is>
-          <t>期末数|期初数</t>
+          <t>本季度数|上季度数</t>
         </is>
       </c>
       <c r="J46" s="12" t="str"/>
-      <c r="K46" s="25" t="inlineStr">
+      <c r="K46" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2831,17 +2831,17 @@
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>SURRENDER_RISK_CAPITAL</t>
+          <t>INSURANCE_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>寿险业务保险风险-退保风险最低资本</t>
+          <t>寿险业务保险风险最低资本合计</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>退保风险最低资本</t>
+          <t>保险风险最低资本合计</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I47" s="12" t="inlineStr">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="J47" s="12" t="str"/>
-      <c r="K47" s="31" t="inlineStr">
+      <c r="K47" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2884,17 +2884,17 @@
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>MARKET_RISK_CAPITAL</t>
+          <t>SURRENDER_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>市场风险-最低资本合计</t>
+          <t>寿险业务保险风险-退保风险最低资本</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>市场风险最低资本合计</t>
+          <t>退保风险最低资本</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>市场风险</t>
+          <t>保险风险</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="H48" s="12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I48" s="12" t="inlineStr">
@@ -2928,7 +2928,7 @@
         </is>
       </c>
       <c r="J48" s="12" t="str"/>
-      <c r="K48" s="25" t="inlineStr">
+      <c r="K48" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2937,17 +2937,17 @@
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>INTEREST_RATE_RISK_CAPITAL</t>
+          <t>MARKET_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>市场风险-利率风险最低资本</t>
+          <t>市场风险-最低资本合计</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>利率风险最低资本</t>
+          <t>市场风险最低资本合计</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="H49" s="12" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I49" s="12" t="inlineStr">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="J49" s="12" t="str"/>
-      <c r="K49" s="31" t="inlineStr">
+      <c r="K49" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2990,17 +2990,17 @@
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>EQUITY_RISK_CAPITAL</t>
+          <t>INTEREST_RATE_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>市场风险-权益价格风险最低资本</t>
+          <t>市场风险-利率风险最低资本</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>权益价格风险最低资本</t>
+          <t>利率风险最低资本</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -3034,7 +3034,7 @@
         </is>
       </c>
       <c r="J50" s="12" t="str"/>
-      <c r="K50" s="25" t="inlineStr">
+      <c r="K50" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3043,17 +3043,17 @@
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>CREDIT_RISK_CAPITAL</t>
+          <t>EQUITY_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>信用风险-最低资本合计</t>
+          <t>市场风险-权益价格风险最低资本</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>信用风险最低资本合计</t>
+          <t>权益价格风险最低资本</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>信用风险</t>
+          <t>市场风险</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H51" s="12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I51" s="12" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="J51" s="12" t="str"/>
-      <c r="K51" s="31" t="inlineStr">
+      <c r="K51" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3096,17 +3096,17 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>SPREAD_RISK_CAPITAL</t>
+          <t>CREDIT_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>信用风险-利差风险最低资本</t>
+          <t>信用风险-最低资本合计</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>利差风险最低资本</t>
+          <t>信用风险最低资本合计</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="H52" s="12" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I52" s="12" t="inlineStr">
@@ -3140,7 +3140,7 @@
         </is>
       </c>
       <c r="J52" s="12" t="str"/>
-      <c r="K52" s="25" t="inlineStr">
+      <c r="K52" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3149,17 +3149,17 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>COUNTERPARTY_RISK_CAPITAL</t>
+          <t>SPREAD_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>信用风险-交易对手违约风险最低资本</t>
+          <t>信用风险-利差风险最低资本</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>交易对手违约风险最低资本</t>
+          <t>利差风险最低资本</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
@@ -3193,7 +3193,7 @@
         </is>
       </c>
       <c r="J53" s="12" t="str"/>
-      <c r="K53" s="31" t="inlineStr">
+      <c r="K53" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3202,27 +3202,27 @@
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>CASH_LIQUID_ASSETS</t>
+          <t>COUNTERPARTY_RISK_CAPITAL</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>现金及流动性管理工具</t>
+          <t>信用风险-交易对手违约风险最低资本</t>
         </is>
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>现金及流动性管理工具认可价值</t>
+          <t>交易对手违约风险最低资本</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>认可资产</t>
+          <t>最低资本</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>资产构成</t>
+          <t>信用风险</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
@@ -3246,7 +3246,7 @@
         </is>
       </c>
       <c r="J54" s="12" t="str"/>
-      <c r="K54" s="25" t="inlineStr">
+      <c r="K54" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3255,17 +3255,17 @@
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>INVESTMENT_ASSETS</t>
+          <t>CASH_LIQUID_ASSETS</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>投资资产</t>
+          <t>现金及流动性管理工具</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>投资资产认可价值</t>
+          <t>现金及流动性管理工具认可价值</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="H55" s="12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I55" s="12" t="inlineStr">
@@ -3299,7 +3299,7 @@
         </is>
       </c>
       <c r="J55" s="12" t="str"/>
-      <c r="K55" s="31" t="inlineStr">
+      <c r="K55" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3308,17 +3308,17 @@
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>REINSURANCE_ASSETS</t>
+          <t>INVESTMENT_ASSETS</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>再保险资产</t>
+          <t>投资资产</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
-          <t>再保险资产认可价值</t>
+          <t>投资资产认可价值</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="H56" s="12" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I56" s="12" t="inlineStr">
@@ -3352,7 +3352,7 @@
         </is>
       </c>
       <c r="J56" s="12" t="str"/>
-      <c r="K56" s="25" t="inlineStr">
+      <c r="K56" s="31" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3361,27 +3361,27 @@
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>RESERVE_LIABILITIES</t>
+          <t>REINSURANCE_ASSETS</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>准备金负债</t>
+          <t>再保险资产</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>准备金负债认可价值</t>
+          <t>再保险资产认可价值</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>认可负债</t>
+          <t>认可资产</t>
         </is>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>负债构成</t>
+          <t>资产构成</t>
         </is>
       </c>
       <c r="F57" s="12" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="H57" s="12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="I57" s="12" t="inlineStr">
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="J57" s="12" t="str"/>
-      <c r="K57" s="31" t="inlineStr">
+      <c r="K57" s="25" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3414,127 +3414,123 @@
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
         <is>
+          <t>RESERVE_LIABILITIES</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>准备金负债</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>准备金负债认可价值</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>认可负债</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>负债构成</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>期末数|期初数</t>
+        </is>
+      </c>
+      <c r="J58" s="12" t="str"/>
+      <c r="K58" s="31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
           <t>FINANCIAL_LIABILITIES</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>金融负债</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>金融负债认可价值</t>
         </is>
       </c>
-      <c r="D58" s="12" t="inlineStr">
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>认可负债</t>
         </is>
       </c>
-      <c r="E58" s="12" t="inlineStr">
+      <c r="E59" s="12" t="inlineStr">
         <is>
           <t>负债构成</t>
         </is>
       </c>
-      <c r="F58" s="12" t="inlineStr">
-        <is>
-          <t>万元</t>
-        </is>
-      </c>
-      <c r="G58" s="12" t="inlineStr">
-        <is>
-          <t>金额</t>
-        </is>
-      </c>
-      <c r="H58" s="12" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I58" s="12" t="inlineStr">
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="G59" s="12" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I59" s="12" t="inlineStr">
         <is>
           <t>期末数|期初数</t>
         </is>
       </c>
-      <c r="J58" s="12" t="str"/>
-      <c r="K58" s="25" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>FINANCIAL_STATEMENT_ASSETS</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>财务报表资产总额</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>财务报表资产合计</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
-        <is>
-          <t>实际资本</t>
-        </is>
-      </c>
-      <c r="E59" s="13" t="inlineStr">
-        <is>
-          <t>汇总口径</t>
-        </is>
-      </c>
-      <c r="F59" s="13" t="inlineStr">
-        <is>
-          <t>万元</t>
-        </is>
-      </c>
-      <c r="G59" s="13" t="inlineStr">
-        <is>
-          <t>金额</t>
-        </is>
-      </c>
-      <c r="H59" s="13" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I59" s="13" t="inlineStr">
-        <is>
-          <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
-        </is>
-      </c>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
-        </is>
-      </c>
-      <c r="K59" s="31" t="inlineStr">
-        <is>
-          <t>否</t>
+      <c r="J59" s="12" t="str"/>
+      <c r="K59" s="25" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>FINANCIAL_STATEMENT_LIABILITIES</t>
+          <t>FINANCIAL_STATEMENT_ASSETS</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>财务报表负债总额</t>
+          <t>财务报表资产总额</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>财务报表负债合计</t>
+          <t>财务报表资产合计</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
@@ -3572,7 +3568,7 @@
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K60" s="25" t="inlineStr">
+      <c r="K60" s="31" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3581,17 +3577,17 @@
     <row r="61">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>FINANCIAL_STATEMENT_NET_ASSETS</t>
+          <t>FINANCIAL_STATEMENT_LIABILITIES</t>
         </is>
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
-          <t>财务报表净资产总额</t>
+          <t>财务报表负债总额</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>财务报表净资产合计</t>
+          <t>财务报表负债合计</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -3629,7 +3625,7 @@
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K61" s="31" t="inlineStr">
+      <c r="K61" s="25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3638,17 +3634,17 @@
     <row r="62">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>NET_ASSET_ADJUSTMENT</t>
+          <t>FINANCIAL_STATEMENT_NET_ASSETS</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
         <is>
-          <t>对净资产的调整额</t>
+          <t>财务报表净资产总额</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>净资产调整额</t>
+          <t>财务报表净资产合计</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
@@ -3658,7 +3654,7 @@
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>核心一级资本调整</t>
+          <t>汇总口径</t>
         </is>
       </c>
       <c r="F62" s="13" t="inlineStr">
@@ -3686,7 +3682,7 @@
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K62" s="25" t="inlineStr">
+      <c r="K62" s="31" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3695,17 +3691,17 @@
     <row r="63">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>NON_RECOGNIZED_ASSET_BOOK_VALUE</t>
+          <t>NET_ASSET_ADJUSTMENT</t>
         </is>
       </c>
       <c r="B63" s="13" t="inlineStr">
         <is>
-          <t>各项非认可资产的账面价值</t>
+          <t>对净资产的调整额</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>非认可资产账面价值</t>
+          <t>净资产调整额</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
@@ -3743,7 +3739,7 @@
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K63" s="31" t="inlineStr">
+      <c r="K63" s="25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3752,17 +3748,17 @@
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>LONG_TERM_EQUITY_VALUATION_DIFFERENCE</t>
+          <t>NON_RECOGNIZED_ASSET_BOOK_VALUE</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
         <is>
-          <t>长期股权投资的认可价值和账面价值的差额</t>
+          <t>各项非认可资产的账面价值</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>长期股权投资认可价值与账面价值差额|长期股权投资的认可价值与账面价值的差额</t>
+          <t>非认可资产账面价值</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
@@ -3800,7 +3796,7 @@
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K64" s="25" t="inlineStr">
+      <c r="K64" s="31" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3809,17 +3805,17 @@
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>DEFERRED_TAX_ASSET_ADJUSTMENT</t>
+          <t>LONG_TERM_EQUITY_VALUATION_DIFFERENCE</t>
         </is>
       </c>
       <c r="B65" s="13" t="inlineStr">
         <is>
-          <t>递延所得税资产（由经营性亏损引起的递延所得税资产除外）</t>
+          <t>长期股权投资的认可价值和账面价值的差额</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>递延所得税资产(由经营性亏损引起的递延所得税资产除外)</t>
+          <t>长期股权投资认可价值与账面价值差额|长期股权投资的认可价值与账面价值的差额</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
@@ -3857,7 +3853,7 @@
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K65" s="31" t="inlineStr">
+      <c r="K65" s="25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3866,112 +3862,112 @@
     <row r="66">
       <c r="A66" s="13" t="inlineStr">
         <is>
+          <t>DEFERRED_TAX_ASSET_ADJUSTMENT</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>递延所得税资产（由经营性亏损引起的递延所得税资产除外）</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>递延所得税资产(由经营性亏损引起的递延所得税资产除外)</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>实际资本</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t>核心一级资本调整</t>
+        </is>
+      </c>
+      <c r="F66" s="13" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="H66" s="13" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I66" s="13" t="inlineStr">
+        <is>
+          <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
+        </is>
+      </c>
+      <c r="J66" s="13" t="inlineStr">
+        <is>
+          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
+        </is>
+      </c>
+      <c r="K66" s="31" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
           <t>OTHER_CORE_T1_ADJUSTMENT</t>
         </is>
       </c>
-      <c r="B66" s="13" t="inlineStr">
+      <c r="B67" s="13" t="inlineStr">
         <is>
           <t>监管机构规定的其他调整项目</t>
         </is>
       </c>
-      <c r="C66" s="13" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>银保监会规定的其他调整项目|金融监管总局规定的其他调整项目</t>
         </is>
       </c>
-      <c r="D66" s="13" t="inlineStr">
+      <c r="D67" s="13" t="inlineStr">
         <is>
           <t>实际资本</t>
         </is>
       </c>
-      <c r="E66" s="13" t="inlineStr">
+      <c r="E67" s="13" t="inlineStr">
         <is>
           <t>核心一级资本调整</t>
         </is>
       </c>
-      <c r="F66" s="13" t="inlineStr">
-        <is>
-          <t>万元</t>
-        </is>
-      </c>
-      <c r="G66" s="13" t="inlineStr">
-        <is>
-          <t>金额</t>
-        </is>
-      </c>
-      <c r="H66" s="13" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I66" s="13" t="inlineStr">
+      <c r="F67" s="13" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="G67" s="13" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I67" s="13" t="inlineStr">
         <is>
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
-      <c r="J66" s="13" t="inlineStr">
+      <c r="J67" s="13" t="inlineStr">
         <is>
           <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
-      <c r="K66" s="25" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>CORE_T1_INVESTMENT_PROPERTY_FAIR_VALUE_ADJUSTMENT</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>投资性房地产公允价值增值（核心一级资本调整）</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>投资性房地产（包括保险公司以物权方式或通过子公司等方式持有的投资性房地产）的公允价值增值（扣除减值、折旧及所得税影响）</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>实际资本</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>核心一级资本调整</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>万元</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>金额</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
+      <c r="K67" s="25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -3980,12 +3976,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AGRICULTURAL_CATASTROPHE_RISK_RESERVE</t>
+          <t>CORE_T1_INVESTMENT_PROPERTY_FAIR_VALUE_ADJUSTMENT</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>对农业保险提取的大灾风险准备金</t>
+          <t>投资性房地产公允价值增值（核心一级资本调整）</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>投资性房地产（包括保险公司以物权方式或通过子公司等方式持有的投资性房地产）的公允价值增值（扣除减值、折旧及所得税影响）</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4032,12 +4033,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>QUALIFYING_CORE_T1_LIABILITY_CAPITAL</t>
+          <t>AGRICULTURAL_CATASTROPHE_RISK_RESERVE</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>符合核心一级资本标准的负债类资本工具且按规定可计入核心一级资本的金额</t>
+          <t>对农业保险提取的大灾风险准备金</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4084,12 +4085,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>POLICY_SURPLUS_CORE_T1</t>
+          <t>QUALIFYING_CORE_T1_LIABILITY_CAPITAL</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>计入核心一级资本的保单未来盈余</t>
+          <t>符合核心一级资本标准的负债类资本工具且按规定可计入核心一级资本的金额</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4099,7 +4100,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>保单未来盈余</t>
+          <t>核心一级资本调整</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4122,26 +4123,26 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
+        </is>
+      </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CORE_T2_PREFERRED_SHARES</t>
+          <t>POLICY_SURPLUS_CORE_T1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>核心二级资本-优先股</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>优先股</t>
+          <t>计入核心一级资本的保单未来盈余</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4151,7 +4152,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>核心二级资本明细</t>
+          <t>保单未来盈余</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4174,26 +4175,26 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
-        </is>
-      </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>POLICY_SURPLUS_CORE_T2</t>
+          <t>CORE_T2_PREFERRED_SHARES</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>计入核心二级资本的保单未来盈余</t>
+          <t>核心二级资本-优先股</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>优先股</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4203,7 +4204,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>保单未来盈余</t>
+          <t>核心二级资本明细</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -4226,21 +4227,26 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
+        </is>
+      </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>OTHER_CORE_T2_CAPITAL</t>
+          <t>POLICY_SURPLUS_CORE_T2</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>其他核心二级资本</t>
+          <t>计入核心二级资本的保单未来盈余</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4250,7 +4256,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>核心二级资本明细</t>
+          <t>保单未来盈余</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4273,31 +4279,21 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
-        </is>
-      </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CORE_T2_EXCESS_DEDUCTION</t>
+          <t>OTHER_CORE_T2_CAPITAL</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>核心二级资本超限额应扣除部分</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>2.4 减：超限额应扣除的部分</t>
+          <t>其他核心二级资本</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4344,17 +4340,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ANC_T1_SUBORDINATED_TERM_DEBT</t>
+          <t>CORE_T2_EXCESS_DEDUCTION</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>附属一级资本-次级定期债务</t>
+          <t>核心二级资本超限额应扣除部分</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>次级定期债务</t>
+          <t>2.4 减：超限额应扣除的部分</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4364,7 +4360,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>附属一级资本明细</t>
+          <t>核心二级资本明细</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -4401,17 +4397,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ANC_T1_CAPITAL_SUPPLEMENTARY_BONDS</t>
+          <t>ANC_T1_SUBORDINATED_TERM_DEBT</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>附属一级资本-资本补充债券</t>
+          <t>附属一级资本-次级定期债务</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>资本补充债券</t>
+          <t>次级定期债务</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4458,17 +4454,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ANC_T1_CONVERTIBLE_SUBORDINATED_DEBT</t>
+          <t>ANC_T1_CAPITAL_SUPPLEMENTARY_BONDS</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>附属一级资本-可转换次级债</t>
+          <t>附属一级资本-资本补充债券</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>可转换次级债</t>
+          <t>资本补充债券</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4515,17 +4511,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ANC_T1_DEFERRED_TAX_ASSET</t>
+          <t>ANC_T1_CONVERTIBLE_SUBORDINATED_DEBT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>附属一级资本-递延所得税资产（由经营性亏损引起的递延所得税资产除外）</t>
+          <t>附属一级资本-可转换次级债</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>3.4 递延所得税资产（由经营性亏损引起的递延所得税资产除外）</t>
+          <t>可转换次级债</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4572,17 +4568,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ANC_T1_INVESTMENT_PROPERTY_FAIR_VALUE</t>
+          <t>ANC_T1_DEFERRED_TAX_ASSET</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>投资性房地产公允价值增值可计入附属一级资本的金额</t>
+          <t>附属一级资本-递延所得税资产（由经营性亏损引起的递延所得税资产除外）</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>投资性房地产（包括保险公司以物权方式或通过子公司等方式持有的投资性房地产）公允价值增值可计入附属一级资本的金额（扣除减值、折旧及所得税影响）</t>
+          <t>3.4 递延所得税资产（由经营性亏损引起的递延所得税资产除外）</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4629,12 +4625,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>POLICY_SURPLUS_ANC_T1</t>
+          <t>ANC_T1_INVESTMENT_PROPERTY_FAIR_VALUE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>计入附属一级资本的保单未来盈余</t>
+          <t>投资性房地产公允价值增值可计入附属一级资本的金额</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>投资性房地产（包括保险公司以物权方式或通过子公司等方式持有的投资性房地产）公允价值增值可计入附属一级资本的金额（扣除减值、折旧及所得税影响）</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4644,7 +4645,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>保单未来盈余</t>
+          <t>附属一级资本明细</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -4667,21 +4668,26 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
+        </is>
+      </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>OTHER_ANC_T1_CAPITAL</t>
+          <t>POLICY_SURPLUS_ANC_T1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>其他附属一级资本</t>
+          <t>计入附属一级资本的保单未来盈余</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4691,7 +4697,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>附属一级资本明细</t>
+          <t>保单未来盈余</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4714,31 +4720,21 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
-        </is>
-      </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ANC_T1_EXCESS_DEDUCTION</t>
+          <t>OTHER_ANC_T1_CAPITAL</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>附属一级资本超限额应扣除部分</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>3.8 减：超限额应扣除的部分</t>
+          <t>其他附属一级资本</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4785,12 +4781,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>EMERGENCY_OTHER_ANC_T2_CAPITAL</t>
+          <t>ANC_T1_EXCESS_DEDUCTION</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>应急资本等其他附属二级资本</t>
+          <t>附属一级资本超限额应扣除部分</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>3.8 减：超限额应扣除的部分</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4800,7 +4801,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>附属二级资本明细</t>
+          <t>附属一级资本明细</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4837,12 +4838,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>POLICY_SURPLUS_ANC_T2</t>
+          <t>EMERGENCY_OTHER_ANC_T2_CAPITAL</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>计入附属二级资本的保单未来盈余</t>
+          <t>应急资本等其他附属二级资本</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4852,7 +4853,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>保单未来盈余</t>
+          <t>附属二级资本明细</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4875,26 +4876,26 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
+        </is>
+      </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ANC_T2_EXCESS_DEDUCTION</t>
+          <t>POLICY_SURPLUS_ANC_T2</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>附属二级资本超限额应扣除部分</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>4.3 减：超限额应扣除的部分</t>
+          <t>计入附属二级资本的保单未来盈余</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4904,7 +4905,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>附属二级资本明细</t>
+          <t>保单未来盈余</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4927,41 +4928,36 @@
           <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
-        </is>
-      </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SUBSIDIARY_JV_ASSOCIATE_EQUITY</t>
+          <t>ANC_T2_EXCESS_DEDUCTION</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>在子公司合营企业和联营企业中的权益</t>
+          <t>附属二级资本超限额应扣除部分</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>在子公司、合营企业和联营企业中的权益|在子公司合营企业和联营企业中的权益认可价值</t>
+          <t>4.3 减：超限额应扣除的部分</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>认可资产</t>
+          <t>实际资本</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>资产构成</t>
+          <t>附属二级资本明细</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4981,29 +4977,34 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>期末数|期初数</t>
+          <t>本季度数|上季度数|期末数|期初数|本季度末数|上季度末数</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>STEP3完整披露指标；不属于STEP5外部宽表转换范围</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RECEIVABLES_AND_PREPAYMENTS</t>
+          <t>SUBSIDIARY_JV_ASSOCIATE_EQUITY</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>应收及预付款项</t>
+          <t>在子公司合营企业和联营企业中的权益</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>应收及预付款项认可价值</t>
+          <t>在子公司、合营企业和联营企业中的权益|在子公司合营企业和联营企业中的权益认可价值</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5045,17 +5046,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>FIXED_ASSETS</t>
+          <t>RECEIVABLES_AND_PREPAYMENTS</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>固定资产</t>
+          <t>应收及预付款项</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>固定资产认可价值</t>
+          <t>应收及预付款项认可价值</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5097,17 +5098,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>LAND_USE_RIGHTS</t>
+          <t>FIXED_ASSETS</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>土地使用权</t>
+          <t>固定资产</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>土地使用权认可价值</t>
+          <t>固定资产认可价值</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5149,17 +5150,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SEPARATE_ACCOUNT_ASSETS</t>
+          <t>LAND_USE_RIGHTS</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>独立账户资产</t>
+          <t>土地使用权</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>独立账户资产认可价值</t>
+          <t>土地使用权认可价值</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5201,50 +5202,102 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
+          <t>SEPARATE_ACCOUNT_ASSETS</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>独立账户资产</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>独立账户资产认可价值</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>认可资产</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>资产构成</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>期末数|期初数</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>OTHER_RECOGNIZED_ASSETS</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>其他认可资产</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>其他认可资产认可价值</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>认可资产</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>资产构成</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>万元</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>金额</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>万元</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
         <is>
           <t>期末数|期初数</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
+      <c r="K92" t="inlineStr">
         <is>
           <t>是</t>
         </is>

</xml_diff>